<commit_message>
NPB自動更新(1軍): 2026-09-19 (steps: all)
</commit_message>
<xml_diff>
--- a/data/プロ野球/2026年/1軍/レギュラーシーズン/raw/2026-09-19/highlights_20260919.xlsx
+++ b/data/プロ野球/2026年/1軍/レギュラーシーズン/raw/2026-09-19/highlights_20260919.xlsx
@@ -489,7 +489,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>7回表に勝ち越しの2ランホームランを放ち、接戦を制する一打となった。</t>
+          <t>7回表に勝ち越し2ランホームランを放ち、試合の主導権を奪い返した。</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1回と3回にホームランを放ち、1試合2本塁打の活躍でチームを牽引した。</t>
+          <t>先制弾を含む2本塁打を放ち、打線の中核としてチームを牽引した。</t>
         </is>
       </c>
     </row>
@@ -529,17 +529,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>宗 佑磨</t>
+          <t>栗林 良吏</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>オリックス</t>
+          <t>広島</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>6回表に逆転の2ランホームランを放ち、試合の流れを大きく引き寄せた。</t>
+          <t>7回2/3を1失点に抑える好投で、試合の流れを完全に支配した。</t>
         </is>
       </c>
     </row>
@@ -554,17 +554,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>栗林 良吏</t>
+          <t>田中 将大</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>広島</t>
+          <t>巨人</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>7回2/3を1失点に抑える好投で試合を作り、チームの勝利に貢献した。</t>
+          <t>7回を投げ1失点と安定したピッチングで、チームの勝利に貢献した。</t>
         </is>
       </c>
     </row>
@@ -579,17 +579,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>田宮 裕涼</t>
+          <t>宗 佑磨</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>日本ハム</t>
+          <t>オリックス</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4回裏に同点2ランホームランを放ち、試合を振り出しに戻す重要な一打となった。</t>
+          <t>6回表に逆転2ランホームランを放ち、試合の流れを大きく変えた。</t>
         </is>
       </c>
     </row>

</xml_diff>